<commit_message>
feat: hapus panel Lampiran BOQ SPK dari input
</commit_message>
<xml_diff>
--- a/Lampiran BAKH.xlsx
+++ b/Lampiran BAKH.xlsx
@@ -9,10 +9,10 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500" activeTab="3"/>
+    <workbookView windowWidth="15540" windowHeight="7500"/>
   </bookViews>
   <sheets>
-    <sheet name="Format" sheetId="1" r:id="rId1"/>
+    <sheet name="Format bakh" sheetId="1" r:id="rId1"/>
     <sheet name="RAB TA" sheetId="2" r:id="rId2"/>
     <sheet name="RAB MANDOR" sheetId="3" r:id="rId3"/>
     <sheet name="RAB NEGO " sheetId="4" r:id="rId4"/>

</xml_diff>